<commit_message>
fix: nombres de carpetas en minuscula
</commit_message>
<xml_diff>
--- a/data/catalogo_productos.xlsx
+++ b/data/catalogo_productos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://manpowergroupapps-my.sharepoint.com/personal/andres_betancury_manpowergroup_com_co/Documents/1. Proyectos/Cientifico de datos/Pruebas y ejemplos/dk/Mimitos/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_05A231AE924C45E89FBA9C1BDB1CCF0AD6CEE74D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF9AD8CC-22FB-41FD-B8C1-15CA309FB675}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_05A231AE924C45E89FBA9C1BDB1CCF0AD6CEE74D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{789A29C0-D6B3-4766-B7AA-5BE7FDD50FBA}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1288,6 +1288,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="13.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
correccion bug de imagen
</commit_message>
<xml_diff>
--- a/data/catalogo_productos.xlsx
+++ b/data/catalogo_productos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ndrsb\Documents\Mimitos\Mimitos\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{735280F6-6560-487C-869E-3AEF382133DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E24B8BD-877D-4E11-A076-AD16CEE1B191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1694,9 +1694,6 @@
     <t>img/llaveros/k45.jpeg</t>
   </si>
   <si>
-    <t>img/llaveros/k46.jpeg</t>
-  </si>
-  <si>
     <t>img/llaveros/k47.jpeg</t>
   </si>
   <si>
@@ -2358,6 +2355,9 @@
   </si>
   <si>
     <t>img/didacticos/d16.jpeg;img/didacticos/d16_1.jpeg;img/didacticos/d16_2.jpeg</t>
+  </si>
+  <si>
+    <t>img/llaveros/k46.jpeg;img/llaveros/k46_2.jpeg</t>
   </si>
 </sst>
 </file>
@@ -4095,7 +4095,7 @@
         <v>219</v>
       </c>
       <c r="B47" t="s">
-        <v>551</v>
+        <v>772</v>
       </c>
       <c r="C47" t="s">
         <v>76</v>
@@ -4124,7 +4124,7 @@
         <v>219</v>
       </c>
       <c r="B48" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="C48" t="s">
         <v>81</v>
@@ -4153,7 +4153,7 @@
         <v>219</v>
       </c>
       <c r="B49" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="C49" t="s">
         <v>85</v>
@@ -4182,7 +4182,7 @@
         <v>219</v>
       </c>
       <c r="B50" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="C50" t="s">
         <v>90</v>
@@ -4211,7 +4211,7 @@
         <v>219</v>
       </c>
       <c r="B51" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C51" t="s">
         <v>95</v>
@@ -4240,7 +4240,7 @@
         <v>219</v>
       </c>
       <c r="B52" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="C52" t="s">
         <v>99</v>
@@ -4269,7 +4269,7 @@
         <v>219</v>
       </c>
       <c r="B53" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C53" t="s">
         <v>76</v>
@@ -4298,7 +4298,7 @@
         <v>219</v>
       </c>
       <c r="B54" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C54" t="s">
         <v>81</v>
@@ -4327,7 +4327,7 @@
         <v>219</v>
       </c>
       <c r="B55" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="C55" t="s">
         <v>85</v>
@@ -4356,7 +4356,7 @@
         <v>219</v>
       </c>
       <c r="B56" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C56" t="s">
         <v>90</v>
@@ -4386,7 +4386,7 @@
         <v>219</v>
       </c>
       <c r="B57" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C57" t="s">
         <v>95</v>
@@ -4415,7 +4415,7 @@
         <v>220</v>
       </c>
       <c r="B58" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="C58" t="s">
         <v>119</v>
@@ -4444,7 +4444,7 @@
         <v>220</v>
       </c>
       <c r="B59" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="C59" t="s">
         <v>124</v>
@@ -4476,7 +4476,7 @@
         <v>220</v>
       </c>
       <c r="B60" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="C60" t="s">
         <v>129</v>
@@ -4505,7 +4505,7 @@
         <v>220</v>
       </c>
       <c r="B61" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="C61" t="s">
         <v>134</v>
@@ -4537,7 +4537,7 @@
         <v>220</v>
       </c>
       <c r="B62" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="C62" t="s">
         <v>139</v>
@@ -4566,7 +4566,7 @@
         <v>220</v>
       </c>
       <c r="B63" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="C63" t="s">
         <v>144</v>
@@ -4598,7 +4598,7 @@
         <v>220</v>
       </c>
       <c r="B64" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C64" t="s">
         <v>149</v>
@@ -4627,7 +4627,7 @@
         <v>220</v>
       </c>
       <c r="B65" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="C65" t="s">
         <v>154</v>
@@ -4656,7 +4656,7 @@
         <v>220</v>
       </c>
       <c r="B66" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="C66" t="s">
         <v>159</v>
@@ -4685,7 +4685,7 @@
         <v>220</v>
       </c>
       <c r="B67" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="C67" t="s">
         <v>164</v>
@@ -4714,7 +4714,7 @@
         <v>220</v>
       </c>
       <c r="B68" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="C68" t="s">
         <v>169</v>
@@ -4743,7 +4743,7 @@
         <v>220</v>
       </c>
       <c r="B69" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="C69" t="s">
         <v>174</v>
@@ -4775,7 +4775,7 @@
         <v>220</v>
       </c>
       <c r="B70" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="C70" t="s">
         <v>179</v>
@@ -4804,7 +4804,7 @@
         <v>220</v>
       </c>
       <c r="B71" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C71" t="s">
         <v>184</v>
@@ -4833,7 +4833,7 @@
         <v>220</v>
       </c>
       <c r="B72" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C72" t="s">
         <v>189</v>
@@ -4862,7 +4862,7 @@
         <v>220</v>
       </c>
       <c r="B73" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="C73" t="s">
         <v>194</v>
@@ -4891,7 +4891,7 @@
         <v>220</v>
       </c>
       <c r="B74" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="C74" t="s">
         <v>199</v>
@@ -4923,7 +4923,7 @@
         <v>220</v>
       </c>
       <c r="B75" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="C75" t="s">
         <v>204</v>
@@ -4952,7 +4952,7 @@
         <v>220</v>
       </c>
       <c r="B76" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="C76" t="s">
         <v>209</v>
@@ -4981,7 +4981,7 @@
         <v>220</v>
       </c>
       <c r="B77" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="C77" t="s">
         <v>214</v>
@@ -5016,7 +5016,7 @@
         <v>337</v>
       </c>
       <c r="C78" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="D78">
         <v>20000</v>
@@ -5031,13 +5031,13 @@
         <v>11</v>
       </c>
       <c r="H78" t="s">
+        <v>562</v>
+      </c>
+      <c r="I78" t="s">
         <v>563</v>
       </c>
-      <c r="I78" t="s">
+      <c r="J78" t="s">
         <v>564</v>
-      </c>
-      <c r="J78" t="s">
-        <v>565</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
@@ -5048,7 +5048,7 @@
         <v>338</v>
       </c>
       <c r="C79" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="D79">
         <v>800</v>
@@ -5063,13 +5063,13 @@
         <v>47</v>
       </c>
       <c r="H79" t="s">
+        <v>566</v>
+      </c>
+      <c r="I79" t="s">
         <v>567</v>
       </c>
-      <c r="I79" t="s">
-        <v>568</v>
-      </c>
       <c r="J79" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
@@ -5080,7 +5080,7 @@
         <v>339</v>
       </c>
       <c r="C80" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="D80">
         <v>2000</v>
@@ -5092,10 +5092,10 @@
         <v>1</v>
       </c>
       <c r="H80" t="s">
+        <v>569</v>
+      </c>
+      <c r="J80" t="s">
         <v>570</v>
-      </c>
-      <c r="J80" t="s">
-        <v>571</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
@@ -5106,7 +5106,7 @@
         <v>340</v>
       </c>
       <c r="C81" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D81">
         <v>12000</v>
@@ -5118,13 +5118,13 @@
         <v>1</v>
       </c>
       <c r="H81" t="s">
+        <v>572</v>
+      </c>
+      <c r="I81" t="s">
         <v>573</v>
       </c>
-      <c r="I81" t="s">
+      <c r="J81" t="s">
         <v>574</v>
-      </c>
-      <c r="J81" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>341</v>
       </c>
       <c r="C82" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="D82">
         <v>12000</v>
@@ -5147,13 +5147,13 @@
         <v>1</v>
       </c>
       <c r="H82" t="s">
+        <v>572</v>
+      </c>
+      <c r="I82" t="s">
         <v>573</v>
       </c>
-      <c r="I82" t="s">
+      <c r="J82" t="s">
         <v>574</v>
-      </c>
-      <c r="J82" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
@@ -5164,7 +5164,7 @@
         <v>342</v>
       </c>
       <c r="C83" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D83">
         <v>12000</v>
@@ -5176,13 +5176,13 @@
         <v>1</v>
       </c>
       <c r="H83" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I83" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J83" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
@@ -5193,7 +5193,7 @@
         <v>343</v>
       </c>
       <c r="C84" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D84">
         <v>12000</v>
@@ -5205,13 +5205,13 @@
         <v>1</v>
       </c>
       <c r="H84" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I84" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="J84" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
@@ -5222,7 +5222,7 @@
         <v>344</v>
       </c>
       <c r="C85" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="D85">
         <v>12000</v>
@@ -5237,13 +5237,13 @@
         <v>47</v>
       </c>
       <c r="H85" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I85" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="J85" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
@@ -5254,7 +5254,7 @@
         <v>345</v>
       </c>
       <c r="C86" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="D86">
         <v>12000</v>
@@ -5266,13 +5266,13 @@
         <v>1</v>
       </c>
       <c r="H86" t="s">
+        <v>572</v>
+      </c>
+      <c r="I86" t="s">
         <v>573</v>
       </c>
-      <c r="I86" t="s">
+      <c r="J86" t="s">
         <v>574</v>
-      </c>
-      <c r="J86" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
@@ -5283,7 +5283,7 @@
         <v>346</v>
       </c>
       <c r="C87" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="D87">
         <v>12000</v>
@@ -5298,13 +5298,13 @@
         <v>58</v>
       </c>
       <c r="H87" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I87" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="J87" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
@@ -5315,7 +5315,7 @@
         <v>347</v>
       </c>
       <c r="C88" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D88">
         <v>12000</v>
@@ -5327,13 +5327,13 @@
         <v>1</v>
       </c>
       <c r="H88" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I88" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="J88" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
@@ -5344,7 +5344,7 @@
         <v>348</v>
       </c>
       <c r="C89" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="D89">
         <v>12000</v>
@@ -5359,13 +5359,13 @@
         <v>27</v>
       </c>
       <c r="H89" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I89" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="J89" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
@@ -5376,7 +5376,7 @@
         <v>349</v>
       </c>
       <c r="C90" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D90">
         <v>12000</v>
@@ -5388,13 +5388,13 @@
         <v>1</v>
       </c>
       <c r="H90" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I90" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="J90" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
@@ -5405,7 +5405,7 @@
         <v>350</v>
       </c>
       <c r="C91" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D91">
         <v>12000</v>
@@ -5417,13 +5417,13 @@
         <v>1</v>
       </c>
       <c r="H91" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I91" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="J91" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
@@ -5434,7 +5434,7 @@
         <v>351</v>
       </c>
       <c r="C92" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="D92">
         <v>12000</v>
@@ -5446,13 +5446,13 @@
         <v>1</v>
       </c>
       <c r="H92" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I92" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="J92" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
@@ -5463,7 +5463,7 @@
         <v>352</v>
       </c>
       <c r="C93" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="D93">
         <v>12000</v>
@@ -5475,13 +5475,13 @@
         <v>1</v>
       </c>
       <c r="H93" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I93" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="J93" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
@@ -5492,7 +5492,7 @@
         <v>353</v>
       </c>
       <c r="C94" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="D94">
         <v>14000</v>
@@ -5504,13 +5504,13 @@
         <v>1</v>
       </c>
       <c r="H94" t="s">
+        <v>595</v>
+      </c>
+      <c r="I94" t="s">
         <v>596</v>
       </c>
-      <c r="I94" t="s">
-        <v>597</v>
-      </c>
       <c r="J94" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
@@ -5521,7 +5521,7 @@
         <v>354</v>
       </c>
       <c r="C95" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="D95">
         <v>14000</v>
@@ -5533,13 +5533,13 @@
         <v>1</v>
       </c>
       <c r="H95" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="I95" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="J95" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
@@ -5550,7 +5550,7 @@
         <v>355</v>
       </c>
       <c r="C96" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="D96">
         <v>14000</v>
@@ -5562,13 +5562,13 @@
         <v>1</v>
       </c>
       <c r="H96" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="I96" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="J96" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
@@ -5579,7 +5579,7 @@
         <v>356</v>
       </c>
       <c r="C97" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="D97">
         <v>14000</v>
@@ -5594,13 +5594,13 @@
         <v>47</v>
       </c>
       <c r="H97" t="s">
+        <v>595</v>
+      </c>
+      <c r="I97" t="s">
         <v>596</v>
       </c>
-      <c r="I97" t="s">
-        <v>597</v>
-      </c>
       <c r="J97" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
@@ -5611,7 +5611,7 @@
         <v>357</v>
       </c>
       <c r="C98" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D98">
         <v>14000</v>
@@ -5626,13 +5626,13 @@
         <v>27</v>
       </c>
       <c r="H98" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="I98" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="J98" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.25">
@@ -5643,7 +5643,7 @@
         <v>358</v>
       </c>
       <c r="C99" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D99">
         <v>14000</v>
@@ -5655,13 +5655,13 @@
         <v>1</v>
       </c>
       <c r="H99" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="I99" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="J99" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
@@ -5672,7 +5672,7 @@
         <v>359</v>
       </c>
       <c r="C100" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D100">
         <v>35000</v>
@@ -5684,13 +5684,13 @@
         <v>1</v>
       </c>
       <c r="H100" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I100" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="J100" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
@@ -5701,7 +5701,7 @@
         <v>360</v>
       </c>
       <c r="C101" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D101">
         <v>35000</v>
@@ -5713,13 +5713,13 @@
         <v>1</v>
       </c>
       <c r="H101" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I101" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="J101" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
@@ -5730,7 +5730,7 @@
         <v>361</v>
       </c>
       <c r="C102" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D102">
         <v>35000</v>
@@ -5745,13 +5745,13 @@
         <v>47</v>
       </c>
       <c r="H102" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I102" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="J102" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
@@ -5762,7 +5762,7 @@
         <v>362</v>
       </c>
       <c r="C103" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D103">
         <v>35000</v>
@@ -5774,13 +5774,13 @@
         <v>1</v>
       </c>
       <c r="H103" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I103" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="J103" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
@@ -5791,7 +5791,7 @@
         <v>363</v>
       </c>
       <c r="C104" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D104">
         <v>45000</v>
@@ -5803,13 +5803,13 @@
         <v>1</v>
       </c>
       <c r="H104" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I104" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="J104" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.25">
@@ -5820,7 +5820,7 @@
         <v>364</v>
       </c>
       <c r="C105" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D105">
         <v>45000</v>
@@ -5832,13 +5832,13 @@
         <v>1</v>
       </c>
       <c r="H105" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I105" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="J105" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.25">
@@ -5849,7 +5849,7 @@
         <v>365</v>
       </c>
       <c r="C106" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D106">
         <v>45000</v>
@@ -5861,10 +5861,10 @@
         <v>1</v>
       </c>
       <c r="H106" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I106" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="J106" t="s">
         <v>106</v>
@@ -5878,7 +5878,7 @@
         <v>366</v>
       </c>
       <c r="C107" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D107">
         <v>45000</v>
@@ -5893,10 +5893,10 @@
         <v>11</v>
       </c>
       <c r="H107" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I107" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="J107" t="s">
         <v>107</v>
@@ -5910,7 +5910,7 @@
         <v>367</v>
       </c>
       <c r="C108" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D108">
         <v>30000</v>
@@ -5922,10 +5922,10 @@
         <v>1</v>
       </c>
       <c r="H108" t="s">
+        <v>620</v>
+      </c>
+      <c r="I108" t="s">
         <v>621</v>
-      </c>
-      <c r="I108" t="s">
-        <v>622</v>
       </c>
       <c r="J108" t="s">
         <v>108</v>
@@ -5939,7 +5939,7 @@
         <v>368</v>
       </c>
       <c r="C109" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D109">
         <v>30000</v>
@@ -5954,10 +5954,10 @@
         <v>27</v>
       </c>
       <c r="H109" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I109" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="J109" t="s">
         <v>109</v>
@@ -5971,7 +5971,7 @@
         <v>369</v>
       </c>
       <c r="C110" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D110">
         <v>30000</v>
@@ -5983,10 +5983,10 @@
         <v>1</v>
       </c>
       <c r="H110" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I110" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="J110" t="s">
         <v>110</v>
@@ -6000,7 +6000,7 @@
         <v>370</v>
       </c>
       <c r="C111" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D111">
         <v>30000</v>
@@ -6012,10 +6012,10 @@
         <v>1</v>
       </c>
       <c r="H111" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I111" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="J111" t="s">
         <v>111</v>
@@ -6029,7 +6029,7 @@
         <v>371</v>
       </c>
       <c r="C112" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D112">
         <v>30000</v>
@@ -6041,10 +6041,10 @@
         <v>1</v>
       </c>
       <c r="H112" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I112" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="J112" t="s">
         <v>112</v>
@@ -6058,7 +6058,7 @@
         <v>372</v>
       </c>
       <c r="C113" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D113">
         <v>30000</v>
@@ -6070,10 +6070,10 @@
         <v>1</v>
       </c>
       <c r="H113" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I113" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="J113" t="s">
         <v>113</v>
@@ -6087,7 +6087,7 @@
         <v>373</v>
       </c>
       <c r="C114" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D114">
         <v>30000</v>
@@ -6102,10 +6102,10 @@
         <v>47</v>
       </c>
       <c r="H114" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I114" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="J114" t="s">
         <v>114</v>
@@ -6119,7 +6119,7 @@
         <v>374</v>
       </c>
       <c r="C115" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D115">
         <v>30000</v>
@@ -6131,10 +6131,10 @@
         <v>1</v>
       </c>
       <c r="H115" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I115" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="J115" t="s">
         <v>115</v>
@@ -6148,7 +6148,7 @@
         <v>375</v>
       </c>
       <c r="C116" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D116">
         <v>30000</v>
@@ -6163,10 +6163,10 @@
         <v>11</v>
       </c>
       <c r="H116" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I116" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="J116" t="s">
         <v>116</v>
@@ -6180,7 +6180,7 @@
         <v>376</v>
       </c>
       <c r="C117" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D117">
         <v>30000</v>
@@ -6192,10 +6192,10 @@
         <v>1</v>
       </c>
       <c r="H117" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I117" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="J117" t="s">
         <v>117</v>
@@ -6209,7 +6209,7 @@
         <v>377</v>
       </c>
       <c r="C118" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D118">
         <v>30000</v>
@@ -6221,10 +6221,10 @@
         <v>1</v>
       </c>
       <c r="H118" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I118" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="J118" t="s">
         <v>122</v>
@@ -6238,7 +6238,7 @@
         <v>378</v>
       </c>
       <c r="C119" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D119">
         <v>30000</v>
@@ -6253,10 +6253,10 @@
         <v>47</v>
       </c>
       <c r="H119" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I119" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="J119" t="s">
         <v>127</v>
@@ -6270,7 +6270,7 @@
         <v>379</v>
       </c>
       <c r="C120" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D120">
         <v>30000</v>
@@ -6282,10 +6282,10 @@
         <v>1</v>
       </c>
       <c r="H120" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="I120" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="J120" t="s">
         <v>132</v>
@@ -6299,7 +6299,7 @@
         <v>380</v>
       </c>
       <c r="C121" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D121">
         <v>40000</v>
@@ -6314,10 +6314,10 @@
         <v>11</v>
       </c>
       <c r="H121" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I121" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J121" t="s">
         <v>137</v>
@@ -6331,7 +6331,7 @@
         <v>381</v>
       </c>
       <c r="C122" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="D122">
         <v>25000</v>
@@ -6343,10 +6343,10 @@
         <v>1</v>
       </c>
       <c r="H122" t="s">
+        <v>645</v>
+      </c>
+      <c r="I122" t="s">
         <v>646</v>
-      </c>
-      <c r="I122" t="s">
-        <v>647</v>
       </c>
       <c r="J122" t="s">
         <v>142</v>
@@ -6360,7 +6360,7 @@
         <v>382</v>
       </c>
       <c r="C123" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D123">
         <v>25000</v>
@@ -6375,10 +6375,10 @@
         <v>27</v>
       </c>
       <c r="H123" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="I123" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="J123" t="s">
         <v>147</v>
@@ -6392,7 +6392,7 @@
         <v>383</v>
       </c>
       <c r="C124" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D124">
         <v>25000</v>
@@ -6404,10 +6404,10 @@
         <v>1</v>
       </c>
       <c r="H124" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="I124" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="J124" t="s">
         <v>152</v>
@@ -6421,7 +6421,7 @@
         <v>384</v>
       </c>
       <c r="C125" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D125">
         <v>25000</v>
@@ -6433,10 +6433,10 @@
         <v>1</v>
       </c>
       <c r="H125" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="I125" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="J125" t="s">
         <v>157</v>
@@ -6450,7 +6450,7 @@
         <v>385</v>
       </c>
       <c r="C126" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D126">
         <v>18000</v>
@@ -6462,10 +6462,10 @@
         <v>1</v>
       </c>
       <c r="H126" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I126" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="J126" t="s">
         <v>162</v>
@@ -6479,7 +6479,7 @@
         <v>386</v>
       </c>
       <c r="C127" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D127">
         <v>18000</v>
@@ -6491,10 +6491,10 @@
         <v>1</v>
       </c>
       <c r="H127" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I127" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="J127" t="s">
         <v>167</v>
@@ -6508,7 +6508,7 @@
         <v>387</v>
       </c>
       <c r="C128" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D128">
         <v>18000</v>
@@ -6520,10 +6520,10 @@
         <v>1</v>
       </c>
       <c r="H128" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I128" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="J128" t="s">
         <v>172</v>
@@ -6537,7 +6537,7 @@
         <v>388</v>
       </c>
       <c r="C129" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="D129">
         <v>18000</v>
@@ -6552,10 +6552,10 @@
         <v>47</v>
       </c>
       <c r="H129" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="I129" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="J129" t="s">
         <v>177</v>
@@ -6569,7 +6569,7 @@
         <v>389</v>
       </c>
       <c r="C130" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="D130">
         <v>15000</v>
@@ -6581,10 +6581,10 @@
         <v>1</v>
       </c>
       <c r="H130" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I130" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="J130" t="s">
         <v>182</v>
@@ -6598,7 +6598,7 @@
         <v>390</v>
       </c>
       <c r="C131" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="D131">
         <v>15000</v>
@@ -6610,10 +6610,10 @@
         <v>1</v>
       </c>
       <c r="H131" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I131" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J131" t="s">
         <v>187</v>
@@ -6627,7 +6627,7 @@
         <v>391</v>
       </c>
       <c r="C132" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="D132">
         <v>15000</v>
@@ -6639,10 +6639,10 @@
         <v>1</v>
       </c>
       <c r="H132" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I132" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="J132" t="s">
         <v>192</v>
@@ -6656,7 +6656,7 @@
         <v>392</v>
       </c>
       <c r="C133" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="D133">
         <v>15000</v>
@@ -6668,10 +6668,10 @@
         <v>1</v>
       </c>
       <c r="H133" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I133" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="J133" t="s">
         <v>197</v>
@@ -6685,7 +6685,7 @@
         <v>393</v>
       </c>
       <c r="C134" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="D134">
         <v>15000</v>
@@ -6700,10 +6700,10 @@
         <v>11</v>
       </c>
       <c r="H134" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I134" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="J134" t="s">
         <v>202</v>
@@ -6717,7 +6717,7 @@
         <v>394</v>
       </c>
       <c r="C135" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="D135">
         <v>15000</v>
@@ -6729,10 +6729,10 @@
         <v>1</v>
       </c>
       <c r="H135" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I135" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="J135" t="s">
         <v>207</v>
@@ -6746,7 +6746,7 @@
         <v>395</v>
       </c>
       <c r="C136" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="D136">
         <v>15000</v>
@@ -6758,10 +6758,10 @@
         <v>1</v>
       </c>
       <c r="H136" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I136" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="J136" t="s">
         <v>212</v>
@@ -6775,7 +6775,7 @@
         <v>396</v>
       </c>
       <c r="C137" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="D137">
         <v>15000</v>
@@ -6790,10 +6790,10 @@
         <v>27</v>
       </c>
       <c r="H137" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I137" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="J137" t="s">
         <v>109</v>
@@ -6807,7 +6807,7 @@
         <v>397</v>
       </c>
       <c r="C138" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D138">
         <v>15000</v>
@@ -6819,10 +6819,10 @@
         <v>1</v>
       </c>
       <c r="H138" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I138" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="J138" t="s">
         <v>110</v>
@@ -6836,7 +6836,7 @@
         <v>398</v>
       </c>
       <c r="C139" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D139">
         <v>15000</v>
@@ -6848,10 +6848,10 @@
         <v>1</v>
       </c>
       <c r="H139" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I139" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="J139" t="s">
         <v>111</v>
@@ -6865,7 +6865,7 @@
         <v>399</v>
       </c>
       <c r="C140" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D140">
         <v>15000</v>
@@ -6877,10 +6877,10 @@
         <v>1</v>
       </c>
       <c r="H140" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I140" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="J140" t="s">
         <v>112</v>
@@ -6894,7 +6894,7 @@
         <v>400</v>
       </c>
       <c r="C141" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D141">
         <v>15000</v>
@@ -6906,10 +6906,10 @@
         <v>1</v>
       </c>
       <c r="H141" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I141" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J141" t="s">
         <v>113</v>
@@ -6923,7 +6923,7 @@
         <v>401</v>
       </c>
       <c r="C142" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="D142">
         <v>18000</v>
@@ -6935,10 +6935,10 @@
         <v>1</v>
       </c>
       <c r="H142" t="s">
+        <v>677</v>
+      </c>
+      <c r="I142" t="s">
         <v>678</v>
-      </c>
-      <c r="I142" t="s">
-        <v>679</v>
       </c>
       <c r="J142" t="s">
         <v>114</v>
@@ -6952,7 +6952,7 @@
         <v>402</v>
       </c>
       <c r="C143" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="D143">
         <v>18000</v>
@@ -6964,10 +6964,10 @@
         <v>1</v>
       </c>
       <c r="H143" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="I143" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="J143" t="s">
         <v>115</v>
@@ -6981,7 +6981,7 @@
         <v>403</v>
       </c>
       <c r="C144" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="D144">
         <v>18000</v>
@@ -6993,10 +6993,10 @@
         <v>1</v>
       </c>
       <c r="H144" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="I144" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="J144" t="s">
         <v>116</v>
@@ -7010,7 +7010,7 @@
         <v>404</v>
       </c>
       <c r="C145" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="D145">
         <v>18000</v>
@@ -7022,10 +7022,10 @@
         <v>1</v>
       </c>
       <c r="H145" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="I145" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="J145" t="s">
         <v>117</v>
@@ -7039,7 +7039,7 @@
         <v>405</v>
       </c>
       <c r="C146" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="D146">
         <v>18000</v>
@@ -7051,10 +7051,10 @@
         <v>1</v>
       </c>
       <c r="H146" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="I146" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="J146" t="s">
         <v>122</v>
@@ -7068,7 +7068,7 @@
         <v>406</v>
       </c>
       <c r="C147" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="D147">
         <v>18000</v>
@@ -7080,10 +7080,10 @@
         <v>1</v>
       </c>
       <c r="H147" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="I147" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="J147" t="s">
         <v>127</v>
@@ -7097,7 +7097,7 @@
         <v>407</v>
       </c>
       <c r="C148" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="D148">
         <v>18000</v>
@@ -7109,10 +7109,10 @@
         <v>1</v>
       </c>
       <c r="H148" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="I148" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="J148" t="s">
         <v>132</v>
@@ -7126,7 +7126,7 @@
         <v>408</v>
       </c>
       <c r="C149" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="D149">
         <v>18000</v>
@@ -7138,10 +7138,10 @@
         <v>1</v>
       </c>
       <c r="H149" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="I149" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="J149" t="s">
         <v>137</v>
@@ -7155,7 +7155,7 @@
         <v>409</v>
       </c>
       <c r="C150" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="D150">
         <v>15000</v>
@@ -7167,10 +7167,10 @@
         <v>1</v>
       </c>
       <c r="H150" t="s">
+        <v>692</v>
+      </c>
+      <c r="I150" t="s">
         <v>693</v>
-      </c>
-      <c r="I150" t="s">
-        <v>694</v>
       </c>
       <c r="J150" t="s">
         <v>142</v>
@@ -7184,7 +7184,7 @@
         <v>410</v>
       </c>
       <c r="C151" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="D151">
         <v>25000</v>
@@ -7196,10 +7196,10 @@
         <v>1</v>
       </c>
       <c r="H151" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="I151" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="J151" t="s">
         <v>147</v>
@@ -7213,7 +7213,7 @@
         <v>411</v>
       </c>
       <c r="C152" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="D152">
         <v>15000</v>
@@ -7225,10 +7225,10 @@
         <v>1</v>
       </c>
       <c r="H152" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="I152" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="J152" t="s">
         <v>152</v>
@@ -7242,7 +7242,7 @@
         <v>412</v>
       </c>
       <c r="C153" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="D153">
         <v>15000</v>
@@ -7254,10 +7254,10 @@
         <v>1</v>
       </c>
       <c r="H153" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="I153" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="J153" t="s">
         <v>157</v>
@@ -7271,7 +7271,7 @@
         <v>413</v>
       </c>
       <c r="C154" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="D154">
         <v>25000</v>
@@ -7283,10 +7283,10 @@
         <v>1</v>
       </c>
       <c r="H154" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="I154" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="J154" t="s">
         <v>162</v>
@@ -7300,7 +7300,7 @@
         <v>414</v>
       </c>
       <c r="C155" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="D155">
         <v>20000</v>
@@ -7312,10 +7312,10 @@
         <v>1</v>
       </c>
       <c r="H155" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="I155" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="J155" t="s">
         <v>167</v>
@@ -7329,7 +7329,7 @@
         <v>415</v>
       </c>
       <c r="C156" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="D156">
         <v>20000</v>
@@ -7341,10 +7341,10 @@
         <v>1</v>
       </c>
       <c r="H156" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="I156" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="J156" t="s">
         <v>172</v>
@@ -7358,7 +7358,7 @@
         <v>416</v>
       </c>
       <c r="C157" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="D157">
         <v>15000</v>
@@ -7370,10 +7370,10 @@
         <v>1</v>
       </c>
       <c r="H157" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="I157" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="J157" t="s">
         <v>177</v>
@@ -7387,7 +7387,7 @@
         <v>417</v>
       </c>
       <c r="C158" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="D158">
         <v>25000</v>
@@ -7399,10 +7399,10 @@
         <v>1</v>
       </c>
       <c r="H158" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="I158" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="J158" t="s">
         <v>182</v>
@@ -7416,7 +7416,7 @@
         <v>418</v>
       </c>
       <c r="C159" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="D159">
         <v>25000</v>
@@ -7428,10 +7428,10 @@
         <v>1</v>
       </c>
       <c r="H159" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="I159" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="J159" t="s">
         <v>187</v>
@@ -7445,7 +7445,7 @@
         <v>419</v>
       </c>
       <c r="C160" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="D160">
         <v>25000</v>
@@ -7457,10 +7457,10 @@
         <v>1</v>
       </c>
       <c r="H160" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="I160" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="J160" t="s">
         <v>192</v>
@@ -7474,7 +7474,7 @@
         <v>420</v>
       </c>
       <c r="C161" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D161">
         <v>25000</v>
@@ -7486,10 +7486,10 @@
         <v>1</v>
       </c>
       <c r="H161" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="I161" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="J161" t="s">
         <v>197</v>
@@ -7503,7 +7503,7 @@
         <v>421</v>
       </c>
       <c r="C162" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D162">
         <v>25000</v>
@@ -7515,10 +7515,10 @@
         <v>1</v>
       </c>
       <c r="H162" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="I162" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="J162" t="s">
         <v>202</v>
@@ -7532,7 +7532,7 @@
         <v>422</v>
       </c>
       <c r="C163" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="D163">
         <v>25000</v>
@@ -7544,10 +7544,10 @@
         <v>1</v>
       </c>
       <c r="H163" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="I163" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="J163" t="s">
         <v>207</v>
@@ -7561,7 +7561,7 @@
         <v>423</v>
       </c>
       <c r="C164" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="D164">
         <v>25000</v>
@@ -7573,10 +7573,10 @@
         <v>1</v>
       </c>
       <c r="H164" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="I164" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="J164" t="s">
         <v>212</v>
@@ -7590,7 +7590,7 @@
         <v>424</v>
       </c>
       <c r="C165" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="D165">
         <v>25000</v>
@@ -7602,10 +7602,10 @@
         <v>1</v>
       </c>
       <c r="H165" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="I165" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.25">
@@ -7616,7 +7616,7 @@
         <v>425</v>
       </c>
       <c r="C166" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="D166">
         <v>25000</v>
@@ -7628,10 +7628,10 @@
         <v>1</v>
       </c>
       <c r="H166" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="I166" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.25">
@@ -7642,7 +7642,7 @@
         <v>426</v>
       </c>
       <c r="C167" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="D167">
         <v>25000</v>
@@ -7654,10 +7654,10 @@
         <v>1</v>
       </c>
       <c r="H167" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="I167" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.25">
@@ -7668,7 +7668,7 @@
         <v>427</v>
       </c>
       <c r="C168" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="D168">
         <v>27000</v>
@@ -7680,10 +7680,10 @@
         <v>1</v>
       </c>
       <c r="H168" t="s">
+        <v>719</v>
+      </c>
+      <c r="I168" t="s">
         <v>720</v>
-      </c>
-      <c r="I168" t="s">
-        <v>721</v>
       </c>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.25">
@@ -7694,7 +7694,7 @@
         <v>428</v>
       </c>
       <c r="C169" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="D169">
         <v>27000</v>
@@ -7706,10 +7706,10 @@
         <v>1</v>
       </c>
       <c r="H169" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="I169" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.25">
@@ -7720,7 +7720,7 @@
         <v>429</v>
       </c>
       <c r="C170" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D170">
         <v>27000</v>
@@ -7732,10 +7732,10 @@
         <v>1</v>
       </c>
       <c r="H170" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="I170" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.25">
@@ -7746,7 +7746,7 @@
         <v>430</v>
       </c>
       <c r="C171" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="D171">
         <v>27000</v>
@@ -7758,10 +7758,10 @@
         <v>1</v>
       </c>
       <c r="H171" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="I171" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.25">
@@ -7772,7 +7772,7 @@
         <v>431</v>
       </c>
       <c r="C172" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="D172">
         <v>27000</v>
@@ -7784,10 +7784,10 @@
         <v>1</v>
       </c>
       <c r="H172" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="I172" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.25">
@@ -7798,7 +7798,7 @@
         <v>432</v>
       </c>
       <c r="C173" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="D173">
         <v>27000</v>
@@ -7810,10 +7810,10 @@
         <v>1</v>
       </c>
       <c r="H173" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="I173" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.25">
@@ -7824,7 +7824,7 @@
         <v>433</v>
       </c>
       <c r="C174" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="D174">
         <v>35000</v>
@@ -7836,10 +7836,10 @@
         <v>1</v>
       </c>
       <c r="H174" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="I174" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.25">
@@ -7850,7 +7850,7 @@
         <v>434</v>
       </c>
       <c r="C175" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="D175">
         <v>35000</v>
@@ -7862,10 +7862,10 @@
         <v>1</v>
       </c>
       <c r="H175" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="I175" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.25">
@@ -7876,7 +7876,7 @@
         <v>435</v>
       </c>
       <c r="C176" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D176">
         <v>35000</v>
@@ -7888,10 +7888,10 @@
         <v>1</v>
       </c>
       <c r="H176" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="I176" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
@@ -7902,7 +7902,7 @@
         <v>436</v>
       </c>
       <c r="C177" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="D177">
         <v>35000</v>
@@ -7914,10 +7914,10 @@
         <v>1</v>
       </c>
       <c r="H177" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="I177" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.25">
@@ -7928,7 +7928,7 @@
         <v>437</v>
       </c>
       <c r="C178" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="D178">
         <v>35000</v>
@@ -7940,10 +7940,10 @@
         <v>1</v>
       </c>
       <c r="H178" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="I178" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -7954,7 +7954,7 @@
         <v>438</v>
       </c>
       <c r="C179" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="D179">
         <v>35000</v>
@@ -7966,10 +7966,10 @@
         <v>1</v>
       </c>
       <c r="H179" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="I179" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
@@ -7980,7 +7980,7 @@
         <v>439</v>
       </c>
       <c r="C180" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="D180">
         <v>25000</v>
@@ -7992,10 +7992,10 @@
         <v>1</v>
       </c>
       <c r="H180" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="I180" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -8006,7 +8006,7 @@
         <v>440</v>
       </c>
       <c r="C181" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D181">
         <v>25000</v>
@@ -8018,10 +8018,10 @@
         <v>1</v>
       </c>
       <c r="H181" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="I181" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
@@ -8032,7 +8032,7 @@
         <v>441</v>
       </c>
       <c r="C182" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="D182">
         <v>25000</v>
@@ -8044,10 +8044,10 @@
         <v>1</v>
       </c>
       <c r="H182" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="I182" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
@@ -8058,7 +8058,7 @@
         <v>442</v>
       </c>
       <c r="C183" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="D183">
         <v>25000</v>
@@ -8070,10 +8070,10 @@
         <v>1</v>
       </c>
       <c r="H183" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="I183" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
@@ -8084,7 +8084,7 @@
         <v>443</v>
       </c>
       <c r="C184" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D184">
         <v>25000</v>
@@ -8096,10 +8096,10 @@
         <v>1</v>
       </c>
       <c r="H184" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="I184" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -8110,7 +8110,7 @@
         <v>444</v>
       </c>
       <c r="C185" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="D185">
         <v>15000</v>
@@ -8122,10 +8122,10 @@
         <v>6</v>
       </c>
       <c r="H185" t="s">
+        <v>740</v>
+      </c>
+      <c r="I185" t="s">
         <v>741</v>
-      </c>
-      <c r="I185" t="s">
-        <v>742</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
@@ -8136,7 +8136,7 @@
         <v>445</v>
       </c>
       <c r="C186" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="D186">
         <v>25000</v>
@@ -8148,10 +8148,10 @@
         <v>1</v>
       </c>
       <c r="H186" t="s">
+        <v>743</v>
+      </c>
+      <c r="I186" t="s">
         <v>744</v>
-      </c>
-      <c r="I186" t="s">
-        <v>745</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
@@ -8162,7 +8162,7 @@
         <v>446</v>
       </c>
       <c r="C187" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="D187">
         <v>15000</v>
@@ -8174,10 +8174,10 @@
         <v>1</v>
       </c>
       <c r="H187" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="I187" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.25">
@@ -8188,7 +8188,7 @@
         <v>447</v>
       </c>
       <c r="C188" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="D188">
         <v>15000</v>
@@ -8200,10 +8200,10 @@
         <v>1</v>
       </c>
       <c r="H188" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="I188" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
@@ -8214,7 +8214,7 @@
         <v>448</v>
       </c>
       <c r="C189" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="D189">
         <v>15000</v>
@@ -8226,10 +8226,10 @@
         <v>1</v>
       </c>
       <c r="H189" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="I189" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
@@ -8240,7 +8240,7 @@
         <v>449</v>
       </c>
       <c r="C190" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="D190">
         <v>15000</v>
@@ -8252,10 +8252,10 @@
         <v>1</v>
       </c>
       <c r="H190" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="I190" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
   </sheetData>
@@ -12636,7 +12636,7 @@
         <v>118</v>
       </c>
       <c r="B1" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C1">
         <v>1</v>
@@ -12650,7 +12650,7 @@
         <v>123</v>
       </c>
       <c r="B2" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -12664,7 +12664,7 @@
         <v>128</v>
       </c>
       <c r="B3" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C3">
         <v>3</v>
@@ -12678,7 +12678,7 @@
         <v>133</v>
       </c>
       <c r="B4" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C4">
         <v>4</v>
@@ -12692,7 +12692,7 @@
         <v>138</v>
       </c>
       <c r="B5" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C5">
         <v>5</v>
@@ -12706,7 +12706,7 @@
         <v>143</v>
       </c>
       <c r="B6" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C6">
         <v>6</v>
@@ -12720,7 +12720,7 @@
         <v>148</v>
       </c>
       <c r="B7" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C7">
         <v>7</v>
@@ -12734,7 +12734,7 @@
         <v>153</v>
       </c>
       <c r="B8" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C8">
         <v>8</v>
@@ -12748,7 +12748,7 @@
         <v>158</v>
       </c>
       <c r="B9" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C9">
         <v>9</v>
@@ -12762,7 +12762,7 @@
         <v>163</v>
       </c>
       <c r="B10" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C10">
         <v>10</v>
@@ -12776,7 +12776,7 @@
         <v>168</v>
       </c>
       <c r="B11" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C11">
         <v>11</v>
@@ -12790,7 +12790,7 @@
         <v>173</v>
       </c>
       <c r="B12" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C12">
         <v>12</v>
@@ -12804,7 +12804,7 @@
         <v>178</v>
       </c>
       <c r="B13" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C13">
         <v>13</v>
@@ -12818,7 +12818,7 @@
         <v>183</v>
       </c>
       <c r="B14" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C14">
         <v>14</v>
@@ -12832,7 +12832,7 @@
         <v>188</v>
       </c>
       <c r="B15" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C15">
         <v>15</v>
@@ -12846,7 +12846,7 @@
         <v>193</v>
       </c>
       <c r="B16" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C16">
         <v>16</v>
@@ -12860,7 +12860,7 @@
         <v>198</v>
       </c>
       <c r="B17" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C17">
         <v>17</v>
@@ -12874,7 +12874,7 @@
         <v>203</v>
       </c>
       <c r="B18" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C18">
         <v>18</v>
@@ -12888,7 +12888,7 @@
         <v>208</v>
       </c>
       <c r="B19" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C19">
         <v>19</v>
@@ -12902,7 +12902,7 @@
         <v>213</v>
       </c>
       <c r="B20" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C20">
         <v>20</v>

</xml_diff>